<commit_message>
updated notes on using relative vs absolute paths in the metadata
</commit_message>
<xml_diff>
--- a/Metadata_Template.xlsx
+++ b/Metadata_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/t.brekke/Kew/Fungal_OTU_Sanger/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/t.brekke/Kew/MycorrhizaTracer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74B224C8-EC39-2842-81DC-2CED2CCFE647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C7B06B9-6FCC-E34B-89CB-EC82F935E638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17260" xr2:uid="{BE3650CD-DF03-FA4A-849B-1A75BF225640}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="29400" windowHeight="17260" activeTab="1" xr2:uid="{BE3650CD-DF03-FA4A-849B-1A75BF225640}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -84,9 +84,6 @@
     <t>a grouping factor if you want poor quality sequences to be salvaged. Will only be classified to a species if another sample with the same grouping factor is classified to that speces</t>
   </si>
   <si>
-    <t xml:space="preserve">The directory that the data files are stored in. Can be as long or short as is helpful. Will be combined with the following columns and must create the full file path to the data. </t>
-  </si>
-  <si>
     <t>maybe</t>
   </si>
   <si>
@@ -127,6 +124,9 @@
   </si>
   <si>
     <t>Plot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The directory that the data files are stored in. Can be as long or short as is helpful. Will be combined with --prefix and the following columns and must create the full file path to the data. If you intend to use --prefix then this must not be an absolute path. </t>
   </si>
 </sst>
 </file>
@@ -517,7 +517,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -541,10 +541,10 @@
         <v>7</v>
       </c>
       <c r="J1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -585,7 +585,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
@@ -599,10 +599,10 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -610,10 +610,10 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -621,10 +621,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
@@ -632,10 +632,10 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -643,10 +643,10 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -654,10 +654,10 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -665,26 +665,26 @@
         <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" t="s">
         <v>26</v>
-      </c>
-      <c r="B11" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>